<commit_message>
Ensure date is displayed on fist column on both onboarded Excel files
</commit_message>
<xml_diff>
--- a/data/une_rt_a__custom_14324113_page_spreadsheet.xlsx
+++ b/data/une_rt_a__custom_14324113_page_spreadsheet.xlsx
@@ -608,9 +608,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>9360</xdr:colOff>
+      <xdr:colOff>9000</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>56520</xdr:rowOff>
+      <xdr:rowOff>56160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -624,7 +624,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="12412800" cy="628200"/>
+          <a:ext cx="12412440" cy="627840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1365,7 +1365,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="11.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>14</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="11.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
         <v>64</v>
       </c>

</xml_diff>